<commit_message>
added fact_orders and modified fact order_items and web events
</commit_message>
<xml_diff>
--- a/E-commerce dimensional modelling .xlsx
+++ b/E-commerce dimensional modelling .xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Data projects\data engineering\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{986020C6-4ED7-456E-A911-284349991C99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD59EC13-7F33-4F84-B688-DFDE894FC557}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E0184B5A-05EB-4507-9DC9-AEEFC2718DCA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="75">
   <si>
     <t>dim_customers</t>
   </si>
@@ -125,50 +125,149 @@
     <t>is_weekend</t>
   </si>
   <si>
+    <t>order_id</t>
+  </si>
+  <si>
+    <t>order_date_key</t>
+  </si>
+  <si>
+    <t>currency</t>
+  </si>
+  <si>
+    <t>order_amount_local</t>
+  </si>
+  <si>
+    <t>order_amount_eur</t>
+  </si>
+  <si>
+    <t>quantity</t>
+  </si>
+  <si>
+    <t>fact_web_events</t>
+  </si>
+  <si>
+    <t>event_id</t>
+  </si>
+  <si>
+    <t>session_id</t>
+  </si>
+  <si>
+    <t>event_type</t>
+  </si>
+  <si>
+    <t>page_url</t>
+  </si>
+  <si>
+    <t>event_count</t>
+  </si>
+  <si>
+    <t>Data Model</t>
+  </si>
+  <si>
+    <t>E-Commerce Model</t>
+  </si>
+  <si>
+    <t>Customer</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Order</t>
+  </si>
+  <si>
+    <t>one order</t>
+  </si>
+  <si>
+    <t>Order_Items</t>
+  </si>
+  <si>
+    <t>one product per order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payment </t>
+  </si>
+  <si>
+    <t>one payment</t>
+  </si>
+  <si>
+    <t>Exchange rates</t>
+  </si>
+  <si>
+    <t>one currency rate per day</t>
+  </si>
+  <si>
+    <t>web events</t>
+  </si>
+  <si>
+    <t>one user event</t>
+  </si>
+  <si>
+    <t>Business Processes</t>
+  </si>
+  <si>
+    <t>Grains</t>
+  </si>
+  <si>
+    <t>Bus Matrix</t>
+  </si>
+  <si>
+    <t>Spider/Star Schema</t>
+  </si>
+  <si>
+    <t>dim_currency</t>
+  </si>
+  <si>
+    <t>currency_key</t>
+  </si>
+  <si>
+    <t>currency_id</t>
+  </si>
+  <si>
+    <t>currency_name</t>
+  </si>
+  <si>
+    <t>fact_order_items</t>
+  </si>
+  <si>
+    <t>Fact Table</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Currency</t>
+  </si>
+  <si>
+    <t>Event</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>fact_order_Items</t>
+  </si>
+  <si>
+    <t>dim_prodcucts</t>
+  </si>
+  <si>
+    <t>dim_customer</t>
+  </si>
+  <si>
+    <t>currency attribute</t>
+  </si>
+  <si>
+    <t>dim_product</t>
+  </si>
+  <si>
     <t>fact_orders</t>
-  </si>
-  <si>
-    <t>order_id</t>
-  </si>
-  <si>
-    <t>order_date_key</t>
-  </si>
-  <si>
-    <t>currency</t>
-  </si>
-  <si>
-    <t>order_amount_local</t>
-  </si>
-  <si>
-    <t>order_amount_eur</t>
-  </si>
-  <si>
-    <t>quantity</t>
-  </si>
-  <si>
-    <t>fact_web_events</t>
-  </si>
-  <si>
-    <t>event_id</t>
-  </si>
-  <si>
-    <t>session_id</t>
-  </si>
-  <si>
-    <t>event_type</t>
-  </si>
-  <si>
-    <t>page_url</t>
-  </si>
-  <si>
-    <t>event_count</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -176,19 +275,43 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="1"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -205,6 +328,60 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -221,12 +398,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -244,7 +438,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor theme="1"/>
+          <bgColor theme="4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -262,8 +456,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A2E59BE0-9CC5-47AB-B1A2-1EDBDDFDFC50}" name="Table1" displayName="Table1" ref="B2:B9" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="B2:B9" xr:uid="{A2E59BE0-9CC5-47AB-B1A2-1EDBDDFDFC50}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A2E59BE0-9CC5-47AB-B1A2-1EDBDDFDFC50}" name="Table1" displayName="Table1" ref="C47:C54" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="C47:C54" xr:uid="{A2E59BE0-9CC5-47AB-B1A2-1EDBDDFDFC50}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{FFD054D1-D6D9-461A-89F3-D09E7DA26526}" name="dim_customers"/>
   </tableColumns>
@@ -272,8 +466,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{83AEE5F6-26F0-4417-A637-5CF1F966A0D6}" name="Table2" displayName="Table2" ref="D2:D9" totalsRowShown="0">
-  <autoFilter ref="D2:D9" xr:uid="{83AEE5F6-26F0-4417-A637-5CF1F966A0D6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{83AEE5F6-26F0-4417-A637-5CF1F966A0D6}" name="Table2" displayName="Table2" ref="E47:E54" totalsRowShown="0">
+  <autoFilter ref="E47:E54" xr:uid="{83AEE5F6-26F0-4417-A637-5CF1F966A0D6}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{25512F24-803F-4EF8-A5B9-1BF71A90803E}" name="dim_products"/>
   </tableColumns>
@@ -282,8 +476,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CD6611A0-FCAA-4C70-9156-D8470425DBEC}" name="Table3" displayName="Table3" ref="O5:O16" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="O5:O16" xr:uid="{CD6611A0-FCAA-4C70-9156-D8470425DBEC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CD6611A0-FCAA-4C70-9156-D8470425DBEC}" name="Table3" displayName="Table3" ref="N45:N56" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="N45:N56" xr:uid="{CD6611A0-FCAA-4C70-9156-D8470425DBEC}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{35C8FEAB-119C-4DDB-84AE-9134C6FACFA1}" name="dim_date"/>
   </tableColumns>
@@ -292,10 +486,10 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{968F9B1A-2259-4BEC-9BB3-B901C5C58CB7}" name="Table4" displayName="Table4" ref="G4:H12" totalsRowShown="0">
-  <autoFilter ref="G4:H12" xr:uid="{968F9B1A-2259-4BEC-9BB3-B901C5C58CB7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{968F9B1A-2259-4BEC-9BB3-B901C5C58CB7}" name="Table4" displayName="Table4" ref="G44:H52" totalsRowShown="0">
+  <autoFilter ref="G44:H52" xr:uid="{968F9B1A-2259-4BEC-9BB3-B901C5C58CB7}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{39631442-F523-443F-A7E4-438D75694895}" name="fact_orders"/>
+    <tableColumn id="1" xr3:uid="{39631442-F523-443F-A7E4-438D75694895}" name="fact_order_items"/>
     <tableColumn id="2" xr3:uid="{0225C977-0428-4804-9BAA-CE426BEBE9E7}" name="Column1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -303,8 +497,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{74957C40-0A99-4001-996E-2C866D4C3462}" name="Table5" displayName="Table5" ref="J4:K12" totalsRowShown="0">
-  <autoFilter ref="J4:K12" xr:uid="{74957C40-0A99-4001-996E-2C866D4C3462}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{74957C40-0A99-4001-996E-2C866D4C3462}" name="Table5" displayName="Table5" ref="J44:K52" totalsRowShown="0">
+  <autoFilter ref="J44:K52" xr:uid="{74957C40-0A99-4001-996E-2C866D4C3462}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{A1103E86-AE39-493F-A2B4-F705AF80B768}" name="fact_web_events"/>
     <tableColumn id="2" xr3:uid="{392DDF8A-A39A-468D-A21F-EC2BDCED9CD2}" name="Column1"/>
@@ -630,7 +824,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD9E91E1-B2DF-4111-9FE3-6E82ED79C4A6}">
-  <dimension ref="B2:O16"/>
+  <dimension ref="A1:N68"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="15.7265625" customWidth="1"/>
@@ -643,188 +837,400 @@
     <col min="11" max="11" width="10.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B2" s="1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="8"/>
+      <c r="C3" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" s="12"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" s="12"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="G12" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="H12" s="10"/>
+    </row>
+    <row r="18" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F18" t="s">
+        <v>70</v>
+      </c>
+      <c r="H18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="G19" s="16" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F20" t="s">
+        <v>72</v>
+      </c>
+      <c r="H20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="27" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F27" t="s">
+        <v>71</v>
+      </c>
+      <c r="H27" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="G28" s="17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="30" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="G30" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="39" spans="3:14" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="G39" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="44" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="G44" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="H44" t="s">
+        <v>8</v>
+      </c>
+      <c r="J44" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="K44" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="G45" t="s">
+        <v>29</v>
+      </c>
+      <c r="J45" t="s">
+        <v>36</v>
+      </c>
+      <c r="N45" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="46" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="G46" t="s">
+        <v>1</v>
+      </c>
+      <c r="J46" t="s">
+        <v>18</v>
+      </c>
+      <c r="N46" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="47" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C47" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E47" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B3" t="s">
+      <c r="G47" t="s">
+        <v>10</v>
+      </c>
+      <c r="J47" t="s">
         <v>1</v>
       </c>
-      <c r="D3" t="s">
+      <c r="N47" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="48" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C48" t="s">
+        <v>1</v>
+      </c>
+      <c r="E48" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B4" t="s">
+      <c r="G48" t="s">
+        <v>30</v>
+      </c>
+      <c r="J48" t="s">
+        <v>10</v>
+      </c>
+      <c r="N48" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="49" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C49" t="s">
         <v>2</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E49" t="s">
         <v>11</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="H4" t="s">
-        <v>8</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="K4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B5" t="s">
+      <c r="G49" t="s">
+        <v>31</v>
+      </c>
+      <c r="J49" t="s">
+        <v>37</v>
+      </c>
+      <c r="N49" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="50" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C50" t="s">
         <v>3</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E50" t="s">
         <v>12</v>
       </c>
-      <c r="G5" t="s">
-        <v>30</v>
-      </c>
-      <c r="J5" t="s">
-        <v>37</v>
-      </c>
-      <c r="O5" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B6" t="s">
+      <c r="G50" t="s">
+        <v>32</v>
+      </c>
+      <c r="J50" t="s">
+        <v>38</v>
+      </c>
+      <c r="N50" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="51" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C51" t="s">
         <v>4</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E51" t="s">
         <v>13</v>
       </c>
-      <c r="G6" t="s">
-        <v>1</v>
-      </c>
-      <c r="J6" t="s">
-        <v>18</v>
-      </c>
-      <c r="O6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B7" t="s">
+      <c r="G51" t="s">
+        <v>33</v>
+      </c>
+      <c r="J51" t="s">
+        <v>39</v>
+      </c>
+      <c r="N51" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="52" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C52" t="s">
         <v>5</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E52" t="s">
         <v>15</v>
       </c>
-      <c r="G7" t="s">
-        <v>10</v>
-      </c>
-      <c r="J7" t="s">
-        <v>1</v>
-      </c>
-      <c r="O7" t="s">
+      <c r="G52" t="s">
+        <v>34</v>
+      </c>
+      <c r="J52" t="s">
+        <v>40</v>
+      </c>
+      <c r="N52" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="53" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C53" t="s">
+        <v>6</v>
+      </c>
+      <c r="E53" t="s">
+        <v>14</v>
+      </c>
+      <c r="N53" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="54" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="C54" t="s">
+        <v>7</v>
+      </c>
+      <c r="E54" t="s">
+        <v>16</v>
+      </c>
+      <c r="N54" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="55" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="N55" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="56" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="N56" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="57" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="G57" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="58" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="G58" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="59" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="F59" s="9"/>
+      <c r="G59" s="9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="60" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="G60" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="61" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="G61" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="62" spans="3:14" x14ac:dyDescent="0.35">
+      <c r="G62" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" t="s">
-        <v>14</v>
-      </c>
-      <c r="G8" t="s">
-        <v>31</v>
-      </c>
-      <c r="J8" t="s">
-        <v>10</v>
-      </c>
-      <c r="O8" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" t="s">
-        <v>16</v>
-      </c>
-      <c r="G9" t="s">
-        <v>32</v>
-      </c>
-      <c r="J9" t="s">
-        <v>38</v>
-      </c>
-      <c r="O9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="G10" t="s">
-        <v>33</v>
-      </c>
-      <c r="J10" t="s">
-        <v>39</v>
-      </c>
-      <c r="O10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="G11" t="s">
-        <v>34</v>
-      </c>
-      <c r="J11" t="s">
-        <v>40</v>
-      </c>
-      <c r="O11" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="G12" t="s">
+    <row r="63" spans="3:14" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="D63" s="15" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="65" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C65" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D65" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="E65" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="F65" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="G65" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="H65" s="14" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="66" spans="3:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="C66" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D66" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="E66" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="F66" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="G66" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="H66" s="13"/>
+    </row>
+    <row r="67" spans="3:8" ht="29" x14ac:dyDescent="0.35">
+      <c r="C67" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="J12" t="s">
-        <v>41</v>
-      </c>
-      <c r="O12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="O13" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="O14" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="O15" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="O16" t="s">
-        <v>28</v>
+      <c r="D67" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="E67" s="13"/>
+      <c r="F67" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="G67" s="13"/>
+      <c r="H67" s="13" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="68" spans="3:8" x14ac:dyDescent="0.35">
+      <c r="C68" t="s">
+        <v>74</v>
+      </c>
+      <c r="D68" t="s">
+        <v>68</v>
+      </c>
+      <c r="F68" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="5">
-    <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
     <tablePart r:id="rId5"/>
+    <tablePart r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>